<commit_message>
Minor update for round 1
</commit_message>
<xml_diff>
--- a/docs/Steelhead STARS Elicitation Round 1.xlsx
+++ b/docs/Steelhead STARS Elicitation Round 1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp-my.sharepoint.com/personal/cpien_usbr_gov/Documents/Work/GitHub/steelhead-elicitation/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="59" documentId="8_{B142B1E7-F629-42D5-B6C8-F72BEF73B589}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1A969CD1-CBFA-4FD3-8097-3690A3DFE63F}"/>
+  <xr:revisionPtr revIDLastSave="64" documentId="8_{B142B1E7-F629-42D5-B6C8-F72BEF73B589}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3BBAD9BA-BDA3-49C7-B4A1-AF860EAE507B}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17025" xr2:uid="{7B320B97-FC10-416D-B06B-30ED87F3D6C4}"/>
   </bookViews>
@@ -1516,7 +1516,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0ADA9A65-457B-420C-AF42-0F84516A8CE5}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:AN17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1666,7 +1665,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:40" ht="85.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:40" ht="85.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>45824.438923611109</v>
       </c>
@@ -1749,7 +1748,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:40" ht="210" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:40" ht="210" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>45825.638981481483</v>
       </c>
@@ -2109,7 +2108,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="6" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>45832.464490740742</v>
       </c>
@@ -2213,7 +2212,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="7" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>45832.49554398148</v>
       </c>
@@ -2693,7 +2692,7 @@
       </c>
       <c r="AN10" s="2"/>
     </row>
-    <row r="11" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>45833.493969907409</v>
       </c>
@@ -2809,7 +2808,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>45833.589699074073</v>
       </c>
@@ -2922,7 +2921,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>45833.655243055553</v>
       </c>
@@ -3020,7 +3019,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="14" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>45834.609571759262</v>
       </c>
@@ -3232,7 +3231,7 @@
       <c r="AM15" s="2"/>
       <c r="AN15" s="2"/>
     </row>
-    <row r="16" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>45838.23978009259</v>
       </c>
@@ -3354,7 +3353,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="17" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>45839.460740740738</v>
       </c>
@@ -3474,13 +3473,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AN17" xr:uid="{0ADA9A65-457B-420C-AF42-0F84516A8CE5}">
-    <filterColumn colId="5">
-      <filters>
-        <filter val="Vernalis Flow"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>

</xml_diff>